<commit_message>
Update precipitation monthly title to 'خريطة المتوسط الشهري لتساقط الأمطار (ملم)' across tools, dictionaries, and docs
</commit_message>
<xml_diff>
--- a/docs/Climate_Atlas_Fields_Dictionary_AR_EN_Units.xlsx
+++ b/docs/Climate_Atlas_Fields_Dictionary_AR_EN_Units.xlsx
@@ -1858,7 +1858,7 @@
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>المعدل الشهري لتساقط الأمطار (المتوسط السنوي مقسوماً على 12 شهراً).</t>
+          <t>المتوسط الشهري لتساقط الأمطار (المتوسط السنوي مقسوماً على 12 شهراً).</t>
         </is>
       </c>
       <c r="F36" s="15" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>خريطة المعدل الشهري لتساقط الأمطار (ملم)</t>
+          <t>خريطة المتوسط الشهري لتساقط الأمطار (ملم)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize seasonal precipitation to R_*_Mean across code, GDBs, rasters, and documentation; add interactive HTML filters and complete Arabic documentation
</commit_message>
<xml_diff>
--- a/docs/Climate_Atlas_Fields_Dictionary_AR_EN_Units.xlsx
+++ b/docs/Climate_Atlas_Fields_Dictionary_AR_EN_Units.xlsx
@@ -3025,12 +3025,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>R_WinTot</t>
+          <t>R_WinMean</t>
         </is>
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>R_Winter_Total</t>
+          <t>R_Winter_Mean</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
@@ -3040,17 +3040,17 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>المجموع التراكمي لأمطار فصل الشتاء الأرصادي (شهور ديسمبر، يناير، فبراير - DJF).</t>
+          <t>متوسط هطول الأمطار خلال فصل الشتاء (شهور ديسمبر، يناير، فبراير - DJF).</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>ملم (mm)</t>
+          <t>مم/فصل (mm/season)</t>
         </is>
       </c>
       <c r="G39" s="32" t="inlineStr">
         <is>
-          <t>خريطة مجموع تساقط الأمطار خلال فصل الشتاء (ملم)</t>
+          <t>خريطة متوسط هطول الأمطار خلال فصل الشتاء (مم/فصل)</t>
         </is>
       </c>
     </row>
@@ -3060,12 +3060,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>R_SprTot</t>
+          <t>R_SprMean</t>
         </is>
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
-          <t>R_Spring_Total</t>
+          <t>R_Spring_Mean</t>
         </is>
       </c>
       <c r="D40" s="18" t="inlineStr">
@@ -3075,17 +3075,17 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>المجموع التراكمي لأمطار فصل الربيع الأرصادي (شهور مارس، أبريل، مايو - MAM).</t>
+          <t>متوسط هطول الأمطار خلال فصل الربيع (شهور مارس، أبريل، مايو - MAM).</t>
         </is>
       </c>
       <c r="F40" s="19" t="inlineStr">
         <is>
-          <t>ملم (mm)</t>
+          <t>مم/فصل (mm/season)</t>
         </is>
       </c>
       <c r="G40" s="30" t="inlineStr">
         <is>
-          <t>خريطة مجموع تساقط الأمطار خلال فصل الربيع (ملم)</t>
+          <t>خريطة متوسط هطول الأمطار خلال فصل الربيع (مم/فصل)</t>
         </is>
       </c>
     </row>
@@ -3095,12 +3095,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>R_SumTot</t>
+          <t>R_SumMean</t>
         </is>
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>R_Summer_Total</t>
+          <t>R_Summer_Mean</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -3110,17 +3110,17 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>المجموع التراكمي لأمطار فصل الصيف الأرصادي (شهور يونيو، يوليو، أغسطس - JJA).</t>
+          <t>متوسط هطول الأمطار خلال فصل الصيف (شهور يونيو، يوليو، أغسطس - JJA).</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>ملم (mm)</t>
+          <t>مم/فصل (mm/season)</t>
         </is>
       </c>
       <c r="G41" s="32" t="inlineStr">
         <is>
-          <t>خريطة مجموع تساقط الأمطار خلال فصل الصيف (ملم)</t>
+          <t>خريطة متوسط هطول الأمطار خلال فصل الصيف (مم/فصل)</t>
         </is>
       </c>
     </row>
@@ -3130,12 +3130,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>R_AutTot</t>
+          <t>R_AutMean</t>
         </is>
       </c>
       <c r="C42" s="29" t="inlineStr">
         <is>
-          <t>R_Autumn_Total</t>
+          <t>R_Autumn_Mean</t>
         </is>
       </c>
       <c r="D42" s="18" t="inlineStr">
@@ -3145,17 +3145,17 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>المجموع التراكمي لأمطار فصل الخريف الأرصادي (شهور سبتمبر، أكتوبر، نوفمبر - SON).</t>
+          <t>متوسط هطول الأمطار خلال فصل الخريف (شهور سبتمبر، أكتوبر، نوفمبر - SON).</t>
         </is>
       </c>
       <c r="F42" s="19" t="inlineStr">
         <is>
-          <t>ملم (mm)</t>
+          <t>مم/فصل (mm/season)</t>
         </is>
       </c>
       <c r="G42" s="30" t="inlineStr">
         <is>
-          <t>خريطة مجموع تساقط الأمطار خلال فصل الخريف (ملم)</t>
+          <t>خريطة متوسط هطول الأمطار خلال فصل الخريف (مم/فصل)</t>
         </is>
       </c>
     </row>

</xml_diff>